<commit_message>
new gas turbines can be real peakers
even when gas is not available
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/SuppXLS/Scen_Base_VS.xlsx
+++ b/VerveStacks_ZAF_grids_kan/SuppXLS/Scen_Base_VS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\VerveStacks_ZAF_grids_kan\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5032E83-30B0-48EB-A451-C20EEB42ACED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC8F9214-3A19-4FEE-A89E-4533266874C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grids" sheetId="6" r:id="rId1"/>
@@ -3822,7 +3822,7 @@
         <v>e_w102682082-400_ZAF</v>
       </c>
       <c r="AP5">
-        <f t="shared" ref="AP5:AP68" si="2">4/24</f>
+        <f t="shared" ref="AP5:AP42" si="2">4/24</f>
         <v>0.16666666666666666</v>
       </c>
     </row>
@@ -18866,7 +18866,7 @@
         <v>42</v>
       </c>
       <c r="E27">
-        <v>0.03</v>
+        <v>0.1</v>
       </c>
       <c r="F27" t="str">
         <f>C27</f>

</xml_diff>